<commit_message>
Corri el procesamiento y modelado para argentina nuevamente pero ahora guardando los datos exclusivamente por pais
</commit_message>
<xml_diff>
--- a/modeling/data/argentina/df_modelos.xlsx
+++ b/modeling/data/argentina/df_modelos.xlsx
@@ -455,10 +455,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>92.60618772941794</v>
+        <v>82.18405873099108</v>
       </c>
       <c r="D2" t="n">
-        <v>167.3072570640938</v>
+        <v>135.9256601641918</v>
       </c>
     </row>
     <row r="3">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>93.91714735186156</v>
+        <v>84.49134766649186</v>
       </c>
       <c r="D3" t="n">
-        <v>170.3326896807694</v>
+        <v>139.6043810438838</v>
       </c>
     </row>
     <row r="4">
@@ -497,10 +497,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>94.16622968012587</v>
+        <v>86.43156790770843</v>
       </c>
       <c r="D4" t="n">
-        <v>171.3978443740048</v>
+        <v>146.2115685125011</v>
       </c>
     </row>
     <row r="5">
@@ -513,10 +513,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>74.64604090194021</v>
+        <v>70.00524383848978</v>
       </c>
       <c r="D5" t="n">
-        <v>106.7115029819161</v>
+        <v>95.28236293754347</v>
       </c>
     </row>
     <row r="6">
@@ -529,10 +529,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>81.59412690089145</v>
+        <v>70.64761405348716</v>
       </c>
       <c r="D6" t="n">
-        <v>130.8672322386731</v>
+        <v>98.14028208756929</v>
       </c>
     </row>
     <row r="7">
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>90.87572102779234</v>
+        <v>76.58626114315679</v>
       </c>
       <c r="D7" t="n">
-        <v>161.6580698590597</v>
+        <v>117.4579771771344</v>
       </c>
     </row>
     <row r="8">
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>93.96958573675931</v>
+        <v>87.55899318300996</v>
       </c>
       <c r="D8" t="n">
-        <v>170.6904505617342</v>
+        <v>149.4355157552812</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tras los resultados recien corridos, me doy cuenta que hay algo raro en el procesamiento puesto que la precision promedio con un dataset que nunca vio fue solo del 42%
</commit_message>
<xml_diff>
--- a/modeling/data/argentina/df_modelos.xlsx
+++ b/modeling/data/argentina/df_modelos.xlsx
@@ -455,10 +455,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>82.18405873099108</v>
+        <v>86.14528412419449</v>
       </c>
       <c r="D2" t="n">
-        <v>135.9256601641918</v>
+        <v>148.301630303715</v>
       </c>
     </row>
     <row r="3">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>84.49134766649186</v>
+        <v>89.3526654950205</v>
       </c>
       <c r="D3" t="n">
-        <v>139.6043810438838</v>
+        <v>156.1137900904475</v>
       </c>
     </row>
     <row r="4">
@@ -497,10 +497,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>86.43156790770843</v>
+        <v>90.62683069712946</v>
       </c>
       <c r="D4" t="n">
-        <v>146.2115685125011</v>
+        <v>160.6292165488852</v>
       </c>
     </row>
     <row r="5">
@@ -513,10 +513,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>70.00524383848978</v>
+        <v>73.59402460456943</v>
       </c>
       <c r="D5" t="n">
-        <v>95.28236293754347</v>
+        <v>108.6817244375801</v>
       </c>
     </row>
     <row r="6">
@@ -529,10 +529,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>70.64761405348716</v>
+        <v>74.5459871118922</v>
       </c>
       <c r="D6" t="n">
-        <v>98.14028208756929</v>
+        <v>112.2020817896597</v>
       </c>
     </row>
     <row r="7">
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>76.58626114315679</v>
+        <v>81.57586408904511</v>
       </c>
       <c r="D7" t="n">
-        <v>117.4579771771344</v>
+        <v>134.1693868397511</v>
       </c>
     </row>
     <row r="8">
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>87.55899318300996</v>
+        <v>91.56414762741653</v>
       </c>
       <c r="D8" t="n">
-        <v>149.4355157552812</v>
+        <v>163.4045533971569</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Creo haber encontrado el problema. La precision alta entiendo que es correcta. Sucedia que era baja la precision en el test cuando hacia la separacion de train y test arbitrariamente sin hacer shuffle... Se ve que cuando no hacia shuffle y seleccionaba los ultimos partidos, sacaba los partidos mas recientes y por ende aquellos que son mas importantes puesto que sus datos no son creados artificialmente (sin relleno por tener nan) sino que son reales.
</commit_message>
<xml_diff>
--- a/modeling/data/argentina/df_modelos.xlsx
+++ b/modeling/data/argentina/df_modelos.xlsx
@@ -455,10 +455,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>86.14528412419449</v>
+        <v>76.63099758370728</v>
       </c>
       <c r="D2" t="n">
-        <v>148.301630303715</v>
+        <v>106.6817938003297</v>
       </c>
     </row>
     <row r="3">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>89.3526654950205</v>
+        <v>79.51328960994132</v>
       </c>
       <c r="D3" t="n">
-        <v>156.1137900904475</v>
+        <v>114.9172097478617</v>
       </c>
     </row>
     <row r="4">
@@ -497,10 +497,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>90.62683069712946</v>
+        <v>76.5792198826372</v>
       </c>
       <c r="D4" t="n">
-        <v>160.6292165488852</v>
+        <v>106.7061293198326</v>
       </c>
     </row>
     <row r="5">
@@ -513,10 +513,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>73.59402460456943</v>
+        <v>60.06213324128409</v>
       </c>
       <c r="D5" t="n">
-        <v>108.6817244375801</v>
+        <v>61.94883182308163</v>
       </c>
     </row>
     <row r="6">
@@ -529,10 +529,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>74.5459871118922</v>
+        <v>59.80324473593373</v>
       </c>
       <c r="D6" t="n">
-        <v>112.2020817896597</v>
+        <v>61.18597369398256</v>
       </c>
     </row>
     <row r="7">
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>81.57586408904511</v>
+        <v>75.26751812219538</v>
       </c>
       <c r="D7" t="n">
-        <v>134.1693868397511</v>
+        <v>108.6723012218</v>
       </c>
     </row>
     <row r="8">
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>91.56414762741653</v>
+        <v>76.83810838798757</v>
       </c>
       <c r="D8" t="n">
-        <v>163.4045533971569</v>
+        <v>110.6985352570089</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Las librerias importadas para las pruebas las lleve dentro de la funcion de prueba
</commit_message>
<xml_diff>
--- a/modeling/data/argentina/df_modelos.xlsx
+++ b/modeling/data/argentina/df_modelos.xlsx
@@ -455,10 +455,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>76.63099758370728</v>
+        <v>78.1681497391838</v>
       </c>
       <c r="D2" t="n">
-        <v>106.6817938003297</v>
+        <v>113.306326183763</v>
       </c>
     </row>
     <row r="3">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>79.51328960994132</v>
+        <v>81.60478674440012</v>
       </c>
       <c r="D3" t="n">
-        <v>114.9172097478617</v>
+        <v>117.7882398670104</v>
       </c>
     </row>
     <row r="4">
@@ -497,10 +497,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>76.5792198826372</v>
+        <v>83.26173672905799</v>
       </c>
       <c r="D4" t="n">
-        <v>106.7061293198326</v>
+        <v>124.3615578499184</v>
       </c>
     </row>
     <row r="5">
@@ -513,10 +513,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>60.06213324128409</v>
+        <v>70.69653267873581</v>
       </c>
       <c r="D5" t="n">
-        <v>61.94883182308163</v>
+        <v>87.6195024258663</v>
       </c>
     </row>
     <row r="6">
@@ -529,10 +529,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>59.80324473593373</v>
+        <v>71.80116600184105</v>
       </c>
       <c r="D6" t="n">
-        <v>61.18597369398256</v>
+        <v>89.18890596114133</v>
       </c>
     </row>
     <row r="7">
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>75.26751812219538</v>
+        <v>73.94906413010125</v>
       </c>
       <c r="D7" t="n">
-        <v>108.6723012218</v>
+        <v>99.9849775336242</v>
       </c>
     </row>
     <row r="8">
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>76.83810838798757</v>
+        <v>84.70389690088984</v>
       </c>
       <c r="D8" t="n">
-        <v>110.6985352570089</v>
+        <v>129.0201989169002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corri preparacion y modeling de vuelta para la liga argentina dado que modifique la integracion de datos al implementar + de 1 fecha de actualizacion por fifa
</commit_message>
<xml_diff>
--- a/modeling/data/argentina/df_modelos.xlsx
+++ b/modeling/data/argentina/df_modelos.xlsx
@@ -455,10 +455,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>78.1681497391838</v>
+        <v>80.21761929732564</v>
       </c>
       <c r="D2" t="n">
-        <v>113.306326183763</v>
+        <v>130.7065948817072</v>
       </c>
     </row>
     <row r="3">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>81.60478674440012</v>
+        <v>84.07184058730991</v>
       </c>
       <c r="D3" t="n">
-        <v>117.7882398670104</v>
+        <v>138.649840465643</v>
       </c>
     </row>
     <row r="4">
@@ -497,10 +497,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>83.26173672905799</v>
+        <v>86.44467750393288</v>
       </c>
       <c r="D4" t="n">
-        <v>124.3615578499184</v>
+        <v>146.8817492228531</v>
       </c>
     </row>
     <row r="5">
@@ -513,10 +513,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>70.69653267873581</v>
+        <v>69.67750393287886</v>
       </c>
       <c r="D5" t="n">
-        <v>87.6195024258663</v>
+        <v>96.08553283167313</v>
       </c>
     </row>
     <row r="6">
@@ -529,10 +529,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>71.80116600184105</v>
+        <v>71.05401153644468</v>
       </c>
       <c r="D6" t="n">
-        <v>89.18890596114133</v>
+        <v>101.1019273129745</v>
       </c>
     </row>
     <row r="7">
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>73.94906413010125</v>
+        <v>76.50760356581017</v>
       </c>
       <c r="D7" t="n">
-        <v>99.9849775336242</v>
+        <v>118.0648902821085</v>
       </c>
     </row>
     <row r="8">
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>84.70389690088984</v>
+        <v>87.00839014158365</v>
       </c>
       <c r="D8" t="n">
-        <v>129.0201989169002</v>
+        <v>148.5073290190958</v>
       </c>
     </row>
   </sheetData>

</xml_diff>